<commit_message>
Build SchoolResult v6.9.13 — subject-aware report logic
</commit_message>
<xml_diff>
--- a/source/tests/output/formats.xlsx
+++ b/source/tests/output/formats.xlsx
@@ -477,7 +477,7 @@
         <v>وقت التصدير</v>
       </c>
       <c r="B5" t="str">
-        <v>٢‏/١٠‏/٢٠٢٦، ٣:٥٠:٠٢ م</v>
+        <v>٢‏/١٠‏/٢٠٢٦، ٥:٥٤:٠٥ م</v>
       </c>
     </row>
     <row r="6">
@@ -517,7 +517,7 @@
         <v>الإصدار</v>
       </c>
       <c r="B10" t="str">
-        <v>6.9.5</v>
+        <v>6.9.13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>